<commit_message>
Add automatic host, client and solo test assistant
</commit_message>
<xml_diff>
--- a/docs/testing/SkyCraft-Network-Tests.xlsx
+++ b/docs/testing/SkyCraft-Network-Tests.xlsx
@@ -213,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Start" displayName="Start" ref="A1:C9" headerRowCount="1">
-  <autoFilter ref="A1:C9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Start" displayName="Start" ref="A1:C10" headerRowCount="1">
+  <autoFilter ref="A1:C10"/>
   <tableColumns count="3">
     <tableColumn id="1" name="№"/>
     <tableColumn id="2" name="Ситуация"/>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -728,248 +728,265 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="44" customHeight="1">
+    <row r="2" ht="59" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Существующий SkyCraft работает</t>
+          <t>Автоматические проверки</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Распаковать friend-kit вне игры → Установить обновление.cmd → Проверить сборку.cmd → одиночный HUD/движение.</t>
+          <t>Открыть SkyCraft-Хост.exe, SkyCraft-Клиент.exe или SkyCraft-Без-друга.exe из нового комплекта. Папки определяются автоматически. Полный порядок: docs/YS-AUTOTEST.md. Ниже остаются подробные ручные проверки HUD/блоков/разных условий.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Первый тест с другом</t>
+          <t>Существующий SkyCraft работает</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>В одной LAN — L01. В разных сетях — I01: WAN IP/проброс TCP или доступный IPv6. Адрес получить по вкладке Адрес хоста, не наугад.</t>
+          <t>Распаковать friend-kit вне игры → Установить обновление.cmd → Проверить сборку.cmd → одиночный HUD/движение.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Читать конкретный сценарий</t>
+          <t>Первый тест с другом</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>В Сценарии подробно включить фильтр столбца ID, оставить нужный ID. Там полный порядок с командами и нужным Run ID. Подготовка и Адрес хоста объясняют источники переменных.</t>
+          <t>В одной LAN — L01. В разных сетях — I01: WAN IP/проброс TCP или доступный IPv6. Адрес получить по вкладке Адрес хоста, не наугад.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Ввод команд</t>
+          <t>Читать конкретный сценарий</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>T в Skyrim открывает чат Minecraft; /... вводить там. Команды Get-/Test- вводить в Windows PowerShell. Все подписи ENDPOINT/IP заменить своим значением.</t>
+          <t>В Сценарии подробно включить фильтр столбца ID, оставить нужный ID. Там полный порядок с командами и нужным Run ID. Подготовка и Адрес хоста объясняют источники переменных.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Ввод команд</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>T в Skyrim открывает чат Minecraft; /... вводить там. Команды Get-/Test- вводить в Windows PowerShell. Все подписи ENDPOINT/IP заменить своим значением.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Логи и результат</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Прогоны — наблюдения/метрики, Условия прогонов — адрес/версии/режимы. В конце два ZIP с одним ID. PASS TCP не означает PASS игрового сценария.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Запуск без сети</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Проблема HUD/движения: Собрать отчёт.cmd режим 1. Он соберёт AUTO JSONL; ручной Run ID ещё не нужен.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Где файл настроек</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Сначала вкладка «Файлы и команды», G1–G5. Параметры join/network.* находятся в MINECRAFT\config\skycraft.properties. Пустой join = строка join= без текста после знака =.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Где файл настроек</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Сначала вкладка «Файлы и команды», G1–G5. Параметры join/network.* находятся в MINECRAFT\config\skycraft.properties. Пустой join = строка join= без текста после знака =.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Друг сейчас недоступен</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Вкладка «Без друга»: B0–B10 по порядку. Готовые команды, адреса loopback, пять отчётов и возврат DIRECT. Отдельная HTML: БЕЗ-ДРУГА.html.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Открыть: Файлы и команды</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Подготовка</t>
+          <t>Открыть: Файлы и команды</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Адрес хоста</t>
+          <t>Открыть: Подготовка</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Настройка сети</t>
+          <t>Открыть: Адрес хоста</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Без друга</t>
+          <t>Открыть: Настройка сети</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Шаги</t>
+          <t>Открыть: Без друга</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Матрица</t>
+          <t>Открыть: Шаги</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Сценарии подробно</t>
+          <t>Открыть: Матрица</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Прогоны</t>
+          <t>Открыть: Сценарии подробно</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Условия прогонов</t>
+          <t>Открыть: Прогоны</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Откуда данные</t>
+          <t>Открыть: Условия прогонов</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Открыть: Сбор отчёта</t>
+          <t>Открыть: Откуда данные</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
+          <t>Открыть: Сбор отчёта</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
           <t>Открыть: Разбор сбоя</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -5164,7 +5181,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Проверьте активный JAR по установочному отчёту, один skycraft, версия network.2; английская раскладка и чат T.</t>
+          <t>Проверьте активный JAR по установочному отчёту, один skycraft, версия network.3; английская раскладка и чат T.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -5651,12 +5668,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Каждый участник: закройте обе игры по G2. Если network.2 уже установлен, этот шаг пропустите. Если исходный SkyCraft 0.1.2 работает, запустите «Установить обновление.cmd» из P1; в ответ на запрос вставьте полный путь папки Minecraft из G1. Дождитесь сообщения об успешной установке. Если исходного SkyCraft ещё нет, сначала выполните docs/YS-FRIEND.md из комплекта.</t>
+          <t>Каждый участник: закройте обе игры по G2. Если network.3 уже установлен, этот шаг пропустите. Если исходный SkyCraft 0.1.2 работает, запустите «Установить обновление.cmd» из P1; в ответ на запрос вставьте полный путь папки Minecraft из G1. Дождитесь сообщения об успешной установке. Если исходного SkyCraft ещё нет, сначала выполните docs/YS-FRIEND.md из комплекта.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Старые SkyCraft/e4mc сохранятся в SkyCraft-YS-backups рядом с экземпляром. Настройки и миры сохраняются. Единственный активный JAR SkyCraft имеет версию 0.1.2-ys.network.2; e4mc отсутствует, Fabric API остаётся. Проверка версии и SHA256 — P3.</t>
+          <t>Старые SkyCraft/e4mc сохранятся в SkyCraft-YS-backups рядом с экземпляром. Настройки и миры сохраняются. Единственный активный JAR SkyCraft имеет версию 0.1.2-ys.network.3; e4mc отсутствует, Fabric API остаётся. Проверка версии и SHA256 — P3.</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6413,7 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>1. Распакуйте новый комплект целиком вне Skyrim. Откройте эту инструкцию, таблицу и Блокнот для заметок.
-2. Если network.2 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
+2. Если network.3 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
 3. Выполните G1–G5, включая копии и пять базовых строк G4. Запишите состояние VPN/Cloudflare/zapret; для первого прогона выключите их через интерфейсы программ.
 4. Загрузите тестовое сохранение, проверьте HUD, WASD и камеру. В чате:
 /skycraft debug status</t>
@@ -8074,7 +8091,7 @@
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>1. Распакуйте новый комплект целиком вне Skyrim. Откройте эту инструкцию, таблицу и Блокнот для заметок.
-2. Если network.2 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
+2. Если network.3 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
 3. Выполните G1–G5, включая копии и пять базовых строк G4. Запишите состояние VPN/Cloudflare/zapret; для первого прогона выключите их через интерфейсы программ.
 4. Загрузите тестовое сохранение, проверьте HUD, WASD и камеру. В чате:
 /skycraft debug status</t>
@@ -8218,7 +8235,7 @@
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>1. Распакуйте новый комплект целиком вне Skyrim. Откройте эту инструкцию, таблицу и Блокнот для заметок.
-2. Если network.2 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
+2. Если network.3 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
 3. Выполните G1–G5, включая копии и пять базовых строк G4. Запишите состояние VPN/Cloudflare/zapret; для первого прогона выключите их через интерфейсы программ.
 4. Загрузите тестовое сохранение, проверьте HUD, WASD и камеру. В чате:
 /skycraft debug status</t>
@@ -8329,7 +8346,7 @@
       <c r="D9" s="2" t="inlineStr">
         <is>
           <t>1. Распакуйте новый комплект целиком вне Skyrim. Откройте эту инструкцию, таблицу и Блокнот для заметок.
-2. Если network.2 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
+2. Если network.3 уже установлен, повторная установка не нужна. Запустите «Проверить сборку.cmd»: путь Minecraft из G1, папка с SkyrimSE.exe, затем папка Mods вашего MO2 по подсказкам. Откройте полученный ПРОВЕРКА.txt по пути из программы. FAIL сначала разберите, WARN прочитайте.
 3. Выполните G1–G5, включая копии и пять базовых строк G4. Запишите состояние VPN/Cloudflare/zapret; для первого прогона выключите их через интерфейсы программ.
 4. Загрузите тестовое сохранение, проверьте HUD, WASD и камеру. В чате:
 /skycraft debug status</t>

</xml_diff>